<commit_message>
made final changes to get the city, county, states column
</commit_message>
<xml_diff>
--- a/notes_sample.xlsx
+++ b/notes_sample.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\North_American_Management_Work\compare_book_of_negroes_records\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47C59554-ED3D-4474-BE7E-9729E8125F15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A672CA8-AEAF-4865-AB23-7566CB1B8BA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="46200" yWindow="0" windowWidth="25995" windowHeight="10545" xr2:uid="{03E160C7-0AB3-45D1-A274-4590E81AD2CF}"/>
+    <workbookView xWindow="46230" yWindow="0" windowWidth="25965" windowHeight="10545" xr2:uid="{03E160C7-0AB3-45D1-A274-4590E81AD2CF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,119 +39,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Notes</t>
   </si>
   <si>
-    <t>George Black, 35, (Lt. Col. Isaac). Freed by Lawrence Hartshorne as certified</t>
-  </si>
-  <si>
-    <t>Ann Black, 25, ([Lt. Col. Isaac Allen)]. [Freed by Lawrence Hartshorne as certified.]</t>
-  </si>
-  <si>
-    <t>Reuben, 7, ([Lt. Col. Isaac Allen. [Freed by Lawrence Hartshorne as certified.]</t>
-  </si>
-  <si>
-    <t>Sukey, 5, ([Lt. Col. Isaac Allen]). [Freed by Lawrence Hartshorne as certified.]</t>
-  </si>
-  <si>
-    <t>Billy Williams, 35, healthy stout man, (Richard Browne). Formerly lived with Mr. Moore of Reedy Island, Caroline, from whence he came with the 71st Regiment about 3 years ago.</t>
-  </si>
-  <si>
-    <t>Rose Richard, 20, healthy young woman, (Thomas Richard). Property of Thomas Richard, a refugee from Philadelphia.</t>
-  </si>
-  <si>
-    <t>Daniel Barber, 70, worn out, (James Moore). Says he was made free by Mr. Austin Moore of little York nigh 20 years ago.</t>
-  </si>
-  <si>
-    <t>Sarah Farmer, 23, healthy young woman, (Mrs. Sharp).</t>
-  </si>
-  <si>
-    <t>Barbarry Allen, 22, healthy stout wench, (Humphry Winters). Property of Humphrey Winters of New York from Virginia.</t>
-  </si>
-  <si>
-    <t>Elizabeth Black, 24, mulatto from Madagascar, (Mr. Buskirk). Free, indented when nine years of age to Mrs. Courtland.</t>
-  </si>
-  <si>
-    <t>Bob Stafford, 20, stout healthy Negro, (Mr. Sharp). Taken from Mr. Wilkinson in Virginia by a party from the Royal Navy about four years ago.</t>
-  </si>
-  <si>
-    <t>Harry Covenhoven, 24, [stout healthy Negro], (Mr. Buskirk). Came in two years ago from Mr. Covenhoven in Jersey.</t>
-  </si>
-  <si>
-    <t>John Vans, 39, healthy, blind of his right eye, (Mr. Buskirk, Jr.). Taken in Pennsylvania a party of the British Army about 6½ years ago; lived there with Sam Barber who he says had eight months before given him his freedom.</t>
-  </si>
-  <si>
-    <t>Anthony Haln, 27, stout Negro, (Nicholas Beckle). His own property willed</t>
-  </si>
-  <si>
-    <t>Joyce, 12, healthy Negress, (James Moore). Lived with James Moore for 6 years; her father died in the King's service.</t>
-  </si>
-  <si>
-    <t>Simson McGuire, 223, stout healthy Negro man, (John Buskirk). Came in to General Arnold in Virginia from Benjamin Hill.</t>
-  </si>
-  <si>
-    <t>Bristol Cobbwine, 14, stout healthy Negro boy, (Richard Browne). Came from Woodbury, Charlestown, South Carolina, with Major Grant of the King's American regiment about 4 years ago.</t>
-  </si>
-  <si>
-    <t>Paul, 19, [stout] mulatto, ([Richard Browne]). Came from Woodbury, Charlestown, South Carolina, with Major Grant of the King's American regiment.</t>
-  </si>
-  <si>
-    <t>Sam Brothers, 25, stout Negro man, (Thomas Harrison). Certificate from General Birch formerly lived with Willis Wilkinson in Virginia.</t>
-  </si>
-  <si>
-    <t>Betsy his wife, 2 children, 32, 14 &amp; 12, stout &amp; healthy, ([Thomas Harrison]). Certificate from General Birch, formerly lived with Willis Wilkinson in Virginia.</t>
-  </si>
-  <si>
-    <t>William Mannan, 27, thin lathy fellow, (Richard White). Formerly slave to George Sobriskey at Oldbridge, Jersey, about 7 years ago.</t>
-  </si>
-  <si>
-    <t>Henry McGrigger, 24, stout fellow, (Alpheus Palmer). Formerly slave to Thomas Haywood, Charlestown; joined the British troops under the command of General Provost on its march near Charlestown.</t>
-  </si>
-  <si>
-    <t>Peter Randall, 23, stout fellow, (William Cassels). Formerly slave to James Field in Petersburg, Virginia whom he left 4 years ago &amp; came to New York.</t>
-  </si>
-  <si>
-    <t>Robert Blew, 30, stout fellow, (Richard White). Formerly a servant to Captain Gills who left him with Parson turner which parson he left 4 years ago &amp; joined the British troops at Norfolk in Consequence of Proclamation.</t>
-  </si>
-  <si>
-    <t>Sippio Simmons, 26, stout lad, (Richard White). Given to General Provost by General Haldin and on the General's death left him free.</t>
-  </si>
-  <si>
-    <t>Jacob Miles, 36, stout fellow, (James Dowell). Came with the troops from Philadelphia to New York; says he was born free at Dover, Pennsylvania.</t>
-  </si>
-  <si>
-    <t>Williiam Fortune, 40, stout man, (Mr. Ray). Formerly slave to John Morgan at Harrington, New Jersey, came in on the strength of General Howe's proclamation 6 years past. GBC.</t>
-  </si>
-  <si>
-    <t>Samuel Wyllie, 30, stout man, (Mr. Ray). Formerly slave to Edward Davis at Savannah; left the said place with General Clark and the troops. GBC.</t>
-  </si>
-  <si>
-    <t>Gad Saunders, 25, stout man, (George Rapalje). Formerly slave to David Gilbert, New Haven, Connecticut; left him 4 years ago. Deserter from the Continental army.</t>
-  </si>
-  <si>
-    <t>Judith Saunders, 25, stout wench, better half Indian (George Rapalje). Born free at Stonington in the home of Thomas Williams, Connecticut.</t>
-  </si>
-  <si>
-    <t>Simsa Herring, 25, stout fellow, (Charles Oliver Bruff). Formerly slave to Daniel Herring near Tappan, New Jersey; left 4½ years ago on the strength of the proclamation.</t>
-  </si>
-  <si>
-    <t>Thomas Ogden, 29, stout, scar on the point of left eye, (on his own bottom). Formerly slave to Stephen Baldwin, New Jersey; left him 4½ years ago in consequence of proclamation.</t>
-  </si>
-  <si>
-    <t>Ben Broughton, 38, passable, (Alpheus Palmer). Formerly slave to Thomas Hoggat, Norfolk, Virginia; left him about 4 years ago in consequence of Proclamation.</t>
-  </si>
-  <si>
-    <t>Thomas Smith, 25, stout, brickmaker, (Charles Oliver Bruff). Formerly slave to Sparrows Maybee, Tappan, New Jersey; left him about 5 years ago in consequence of Proclamation.</t>
-  </si>
-  <si>
-    <t>William Bogert, 20, stout make, (Charles Oliver Bruff). Formerly slave to John Bogert, Tappan, New Jersey; left him about 5 years ago in consequence of Proclamation.</t>
-  </si>
-  <si>
-    <t>William Syrrus, 30, stout make, (Alpheus Palmer). Formerly slave to Joseph Smith, Charlestown, taken at the siege of Charlestown on his way from the enemy camp.</t>
-  </si>
-  <si>
     <t>Richard Lautten, 41, stout make, (James Dowell). Free born in New Castle County, Pennsylvania, at his father's house.</t>
   </si>
   <si>
@@ -180,18 +72,6 @@
   </si>
   <si>
     <t>Tom Knight, 38, squat little man, (Joseph Inglish). Left Antigua about four years ago. Steven Clarkely.</t>
-  </si>
-  <si>
-    <t>Moses Palmer, 18, stout, Ben Palmer of Frogs Neck, claimant. Goes with the son Elizabeth Williams, 36, small wench, (Kenneth Renck). Free.</t>
-  </si>
-  <si>
-    <t>Hannah Palmer, 15, stout wench, Ben Palmer of Frogs Neck, claimant. Goes with Ben Palmer's son.</t>
-  </si>
-  <si>
-    <t>Susanna Herring, 22, stout wench, (Charles O. Bruff). Formerly slave to Daniel Herring, Tappan, New Jersey; left him 4½ years past by proclamation.</t>
-  </si>
-  <si>
-    <t>Mary Brown, 38, small wench, (George Rapalje). Formerly slave to Daniel Vancepes, Bergen, New Jersey; left him six years past by proclamation.</t>
   </si>
 </sst>
 </file>
@@ -563,7 +443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{199233EC-55D6-4EA7-9C87-08755FA8ACC3}">
-  <dimension ref="A1:A51"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="255.7109375" bestFit="1" customWidth="1"/>
@@ -624,224 +504,24 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>50</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -989,6 +669,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D83C69F-4358-46DE-BCDA-49E5388EB134}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{42BB06CB-FEE6-46DF-A11E-8CBF95F0C9D6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
@@ -1000,14 +688,6 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D83C69F-4358-46DE-BCDA-49E5388EB134}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
added deepseek integration to get area names
</commit_message>
<xml_diff>
--- a/notes_sample.xlsx
+++ b/notes_sample.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\North_American_Management_Work\compare_book_of_negroes_records\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0835BCF9-08D3-4259-9260-3EA2285779DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{927380AA-09DA-4760-B698-8E22B6536657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="46230" yWindow="10440" windowWidth="25965" windowHeight="10545" xr2:uid="{03E160C7-0AB3-45D1-A274-4590E81AD2CF}"/>
+    <workbookView xWindow="46875" yWindow="0" windowWidth="25320" windowHeight="11025" xr2:uid="{03E160C7-0AB3-45D1-A274-4590E81AD2CF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -54431,12 +54431,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A9F681A11D6F474AB27833CA4A8DFBDD" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ca41a56875ff441cf3dfac098fc17c57">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="77c26180-eae0-4c9b-bc31-a18a32750fb2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5dc1d208de73df6a9cb83d41440df910" ns3:_="">
     <xsd:import namespace="77c26180-eae0-4c9b-bc31-a18a32750fb2"/>
@@ -54580,16 +54589,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D83C69F-4358-46DE-BCDA-49E5388EB134}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{42BB06CB-FEE6-46DF-A11E-8CBF95F0C9D6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
@@ -54605,7 +54613,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C43A102-0E03-4195-8354-86346AC67D3A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -54621,12 +54629,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D83C69F-4358-46DE-BCDA-49E5388EB134}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>